<commit_message>
Fix quote home/away, filtro tornei, matching nomi robusto, pulizia Sackmann
</commit_message>
<xml_diff>
--- a/data/value_bets_log.xlsx
+++ b/data/value_bets_log.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,13 +43,9 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -78,17 +74,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF0000"/>
+        <fgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
     <fill>
@@ -115,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -141,10 +132,7 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -512,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -606,22 +594,22 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>✅ Emiliana Arango</t>
+          <t>✅ Caty McNally</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Linda Noskova</t>
+          <t>Marta Kostyuk</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -635,16 +623,16 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>7.4</v>
+        <v>5.5</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>4.18</v>
+        <v>4.01</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>23.9</v>
+        <v>24.9</v>
       </c>
       <c r="J2" s="6" t="n">
-        <v>76.90000000000001</v>
+        <v>37</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -662,49 +650,49 @@
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>✅ Sergey Fomin</t>
+          <t>✅ Hiroki Moriya</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Andrej Nedic</t>
+          <t>Marat Sharipov</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Challenger - ATP Challenger Shymkent, Kazakhstan Men Singles</t>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>CLAY</t>
+          <t>HARD</t>
         </is>
       </c>
       <c r="G3" s="8" t="n">
-        <v>3.25</v>
+        <v>3.65</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>1.91</v>
+        <v>2.72</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>52.2</v>
+        <v>36.8</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>69.8</v>
+        <v>34.3</v>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>TA-clay</t>
+          <t>TA-hard</t>
         </is>
       </c>
       <c r="L3" s="7" t="inlineStr">
@@ -718,27 +706,27 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>✅ Elena-Gabriela Ruse</t>
+          <t>✅ Laslo Djere</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Elena Rybakina</t>
+          <t>Justin Engel</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>WTA - WTA Madrid, Spain Women Singles</t>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -747,16 +735,16 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>11</v>
+        <v>1.44</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>6.83</v>
+        <v>1.12</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>14.6</v>
+        <v>89.2</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>61</v>
+        <v>28.5</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -774,27 +762,27 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>✅ Stefanos Sakellaridis</t>
+          <t>✅ Coco Gauff</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Jacopo Vasami</t>
+          <t>Linda Noskova</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Challenger - ATP Challenger Rome, Italy Men Singles</t>
+          <t>WTA - WTA Madrid, Spain Women Singles</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -803,16 +791,16 @@
         </is>
       </c>
       <c r="G5" s="8" t="n">
-        <v>1.72</v>
+        <v>1.57</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>1.19</v>
+        <v>1.23</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>83.90000000000001</v>
-      </c>
-      <c r="J5" s="9" t="n">
-        <v>44.3</v>
+        <v>81.2</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>27.5</v>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
@@ -830,27 +818,27 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>✅ Clement Tabur</t>
+          <t>✅ Yusuke Takahashi</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Kilian Feldbausch</t>
+          <t>Yuta Shimizu</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Challenger - ATP Challenger Savannah, USA Men Singles</t>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -859,16 +847,16 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>1.75</v>
+        <v>3.75</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>1.22</v>
+        <v>3.07</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>81.90000000000001</v>
-      </c>
-      <c r="J6" s="9" t="n">
-        <v>43.3</v>
+        <v>32.6</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>22.3</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
@@ -886,22 +874,22 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>✅ Marin Cilic</t>
+          <t>✅ Daniil Medvedev</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Joao Fonseca</t>
+          <t>Nicolai Budkov Kjaer</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -915,16 +903,16 @@
         </is>
       </c>
       <c r="G7" s="8" t="n">
-        <v>4.33</v>
+        <v>1.33</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>3.11</v>
+        <v>1.14</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>32.1</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>39.1</v>
+        <v>16.9</v>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
@@ -942,49 +930,49 @@
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>✅ Nishesh Basavareddy</t>
+          <t>✅ Ann Li</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Andres Andrade</t>
+          <t>Leylah Fernandez</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Challenger - ATP Challenger Savannah, USA Men Singles</t>
+          <t>WTA - WTA Madrid, Spain Women Singles</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>HARD</t>
+          <t>CLAY</t>
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>1.7</v>
+        <v>2.37</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>1.27</v>
+        <v>2.03</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>78.8</v>
+        <v>49.3</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>33.9</v>
+        <v>16.8</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>TA-hard</t>
+          <t>TA-clay</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -998,27 +986,27 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>✅ Sofia Kenin</t>
+          <t>✅ Marco Cecchinato</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Qinwen Zheng</t>
+          <t>Daniel Michalski</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>WTA - WTA Madrid, Spain Women Singles</t>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -1027,16 +1015,16 @@
         </is>
       </c>
       <c r="G9" s="8" t="n">
-        <v>4.33</v>
+        <v>1.57</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>3.31</v>
+        <v>1.35</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>30.2</v>
+        <v>74.3</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>30.9</v>
+        <v>16.6</v>
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
@@ -1054,27 +1042,27 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>✅ Yulia Putintseva</t>
+          <t>✅ Karen Khachanov</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Marta Kostyuk</t>
+          <t>Jakub Mensik</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>WTA - WTA Madrid, Spain Women Singles</t>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1083,16 +1071,16 @@
         </is>
       </c>
       <c r="G10" s="4" t="n">
-        <v>4</v>
+        <v>2.3</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>3.07</v>
+        <v>2</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>32.5</v>
+        <v>49.9</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>30.1</v>
+        <v>14.7</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -1110,49 +1098,49 @@
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>✅ Cameron Norrie</t>
+          <t>✅ Hayato Matsuoka</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Tomas Machac</t>
+          <t>Omar Jasika</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>ATP - ATP Madrid, Spain Men Singles</t>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>CLAY</t>
+          <t>HARD</t>
         </is>
       </c>
       <c r="G11" s="8" t="n">
-        <v>2.12</v>
+        <v>1.66</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>1.66</v>
+        <v>1.45</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>60.1</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>27.4</v>
+        <v>14.7</v>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>TA-clay</t>
+          <t>TA-hard</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr">
@@ -1166,27 +1154,27 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>✅ Andrea Vavassori</t>
+          <t>✅ Tom Gentzsch</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Pol Martin Tiffon</t>
+          <t>George Loffhagen</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Challenger - ATP Challenger Rome, Italy Men Singles</t>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1195,16 +1183,16 @@
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>1.53</v>
+        <v>1.55</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>1.23</v>
+        <v>1.39</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>81.40000000000001</v>
+        <v>71.8</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>24.6</v>
+        <v>11.3</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
@@ -1222,49 +1210,49 @@
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>✅ Linda Klimovicova</t>
+          <t>✅ Karolina Pliskova</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Yue Yuan</t>
+          <t>Solana Sierra</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>WTA 125K - WTA 125K Oeiras 4, Portugal Women Singles</t>
+          <t>WTA - WTA Madrid, Spain Women Singles</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>HARD</t>
+          <t>CLAY</t>
         </is>
       </c>
       <c r="G13" s="8" t="n">
-        <v>2.75</v>
+        <v>1.58</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>2.24</v>
+        <v>1.44</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>44.7</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>22.9</v>
+        <v>10</v>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>TA-hard</t>
+          <t>TA-clay</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
@@ -1278,49 +1266,49 @@
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>✅ Yuta Shimizu</t>
+          <t>✅ Flavio Cobolli</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>August Holmgren</t>
+          <t>Adolfo Daniel Vallejo</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Challenger - ATP Challenger Gwangju, Korea Republic Men Singles</t>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>HARD</t>
+          <t>CLAY</t>
         </is>
       </c>
       <c r="G14" s="4" t="n">
-        <v>2.75</v>
+        <v>1.53</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>2.3</v>
+        <v>1.4</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>43.5</v>
-      </c>
-      <c r="J14" s="10" t="n">
-        <v>19.5</v>
+        <v>71.7</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>9.699999999999999</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>TA-hard</t>
+          <t>TA-clay</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1334,27 +1322,27 @@
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>✅ Leolia Jeanjean</t>
+          <t>✅ Luciano Darderi</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Coco Gauff</t>
+          <t>Francisco Cerundolo</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>WTA - WTA Madrid, Spain Women Singles</t>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -1363,16 +1351,16 @@
         </is>
       </c>
       <c r="G15" s="8" t="n">
-        <v>17</v>
+        <v>2.77</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>14.45</v>
+        <v>2.56</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>6.9</v>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>17.6</v>
+        <v>39</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>8</v>
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
@@ -1390,22 +1378,22 @@
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>✅ Lorenzo Musetti</t>
+          <t>✅ Alexander Zverev</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Hubert Hurkacz</t>
+          <t>Terence Atmane</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1419,16 +1407,16 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>1.54</v>
+        <v>1.17</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>1.31</v>
+        <v>1.11</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>76.2</v>
-      </c>
-      <c r="J16" s="10" t="n">
-        <v>17.3</v>
+        <v>90.09999999999999</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>5.4</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
@@ -1442,790 +1430,6 @@
       </c>
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>✅ Tommy Paul</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>Thiago Agustin Tirante</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>ATP - ATP Madrid, Spain Men Singles</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>CLAY</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="n">
-        <v>1.45</v>
-      </c>
-      <c r="H17" s="5" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="I17" s="7" t="n">
-        <v>80.2</v>
-      </c>
-      <c r="J17" s="10" t="n">
-        <v>16.3</v>
-      </c>
-      <c r="K17" s="7" t="inlineStr">
-        <is>
-          <t>TA-clay</t>
-        </is>
-      </c>
-      <c r="L17" s="7" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M17" s="7" t="inlineStr"/>
-      <c r="N17" s="7" t="inlineStr"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>✅ Katie Boulter</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Jessica Pegula</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>WTA - WTA Madrid, Spain Women Singles</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>CLAY</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="H18" s="5" t="n">
-        <v>5.18</v>
-      </c>
-      <c r="I18" s="2" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="J18" s="10" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>TA-clay</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr"/>
-      <c r="N18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>✅ Gabriel Diallo</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>Elmer Moller</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>ATP - ATP Madrid, Spain Men Singles</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>CLAY</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="n">
-        <v>1.62</v>
-      </c>
-      <c r="H19" s="5" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="I19" s="7" t="n">
-        <v>70.7</v>
-      </c>
-      <c r="J19" s="10" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="K19" s="7" t="inlineStr">
-        <is>
-          <t>TA-clay</t>
-        </is>
-      </c>
-      <c r="L19" s="7" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M19" s="7" t="inlineStr"/>
-      <c r="N19" s="7" t="inlineStr"/>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>✅ Fiona Ferro</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Elena Pridankina</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>WTA 125K - WTA 125K Oeiras 4, Portugal Women Singles</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>HARD</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H20" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="I20" s="2" t="n">
-        <v>66.5</v>
-      </c>
-      <c r="J20" s="10" t="n">
-        <v>13.1</v>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>TA-hard</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="inlineStr"/>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>✅ Cristina Bucsa</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Zeynep Sonmez</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>WTA - WTA Madrid, Spain Women Singles</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>CLAY</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="H21" s="5" t="n">
-        <v>2.22</v>
-      </c>
-      <c r="I21" s="7" t="n">
-        <v>45.1</v>
-      </c>
-      <c r="J21" s="10" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="K21" s="7" t="inlineStr">
-        <is>
-          <t>TA-clay</t>
-        </is>
-      </c>
-      <c r="L21" s="7" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M21" s="7" t="inlineStr"/>
-      <c r="N21" s="7" t="inlineStr"/>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>✅ Arthur Rinderknech</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Dusan Lajovic</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>ATP - ATP Madrid, Spain Men Singles</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>CLAY</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>1.62</v>
-      </c>
-      <c r="H22" s="5" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="I22" s="2" t="n">
-        <v>69.3</v>
-      </c>
-      <c r="J22" s="10" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>TA-clay</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>✅ Sorana Cirstea</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Tyra Caterina Grant</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>WTA - WTA Madrid, Spain Women Singles</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>CLAY</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="H23" s="5" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="I23" s="7" t="n">
-        <v>87.7</v>
-      </c>
-      <c r="J23" s="10" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="K23" s="7" t="inlineStr">
-        <is>
-          <t>TA-clay</t>
-        </is>
-      </c>
-      <c r="L23" s="7" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M23" s="7" t="inlineStr"/>
-      <c r="N23" s="7" t="inlineStr"/>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>✅ Jelena Ostapenko</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Simona Waltert</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>WTA - WTA Madrid, Spain Women Singles</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>CLAY</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="n">
-        <v>1.66</v>
-      </c>
-      <c r="H24" s="5" t="n">
-        <v>1.49</v>
-      </c>
-      <c r="I24" s="2" t="n">
-        <v>67.09999999999999</v>
-      </c>
-      <c r="J24" s="10" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>TA-clay</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>✅ Ben Shelton</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Dino Prizmic</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>ATP - ATP Madrid, Spain Men Singles</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>CLAY</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H25" s="5" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="I25" s="7" t="n">
-        <v>74.2</v>
-      </c>
-      <c r="J25" s="10" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="K25" s="7" t="inlineStr">
-        <is>
-          <t>TA-clay</t>
-        </is>
-      </c>
-      <c r="L25" s="7" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M25" s="7" t="inlineStr"/>
-      <c r="N25" s="7" t="inlineStr"/>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>✅ Elise Mertens</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Alexandra Eala</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>WTA - WTA Madrid, Spain Women Singles</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>CLAY</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="H26" s="5" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="I26" s="2" t="n">
-        <v>78.2</v>
-      </c>
-      <c r="J26" s="2" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>TA-clay</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>✅ Tomas Martin Etcheverry</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>Sebastian Ofner</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>ATP - ATP Madrid, Spain Men Singles</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>CLAY</t>
-        </is>
-      </c>
-      <c r="G27" s="8" t="n">
-        <v>1.61</v>
-      </c>
-      <c r="H27" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="I27" s="7" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="J27" s="7" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="K27" s="7" t="inlineStr">
-        <is>
-          <t>TA-clay</t>
-        </is>
-      </c>
-      <c r="L27" s="7" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M27" s="7" t="inlineStr"/>
-      <c r="N27" s="7" t="inlineStr"/>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>✅ Alex Michelsen</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Jan-Lennard Struff</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>ATP - ATP Madrid, Spain Men Singles</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>CLAY</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="H28" s="5" t="n">
-        <v>2.06</v>
-      </c>
-      <c r="I28" s="2" t="n">
-        <v>48.5</v>
-      </c>
-      <c r="J28" s="2" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="K28" s="2" t="inlineStr">
-        <is>
-          <t>TA-clay</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>✅ Yu Hsiou Hsu</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>Tristan Schoolkate</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>Challenger - ATP Challenger Gwangju, Korea Republic Men Singles</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>HARD</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="n">
-        <v>2.62</v>
-      </c>
-      <c r="H29" s="5" t="n">
-        <v>2.47</v>
-      </c>
-      <c r="I29" s="7" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="J29" s="7" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="K29" s="7" t="inlineStr">
-        <is>
-          <t>TA-hard</t>
-        </is>
-      </c>
-      <c r="L29" s="7" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M29" s="7" t="inlineStr"/>
-      <c r="N29" s="7" t="inlineStr"/>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>03:15</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>✅ Lucia Bronzetti</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>Polina Kudermetova</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>WTA 125K - WTA 125K Oeiras 4, Portugal Women Singles</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>HARD</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="H30" s="5" t="n">
-        <v>3.07</v>
-      </c>
-      <c r="I30" s="2" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="J30" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>TA-hard</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>odds-api.io</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sanity check quote invertite via Elo, dati 2025 TML-Database
</commit_message>
<xml_diff>
--- a/data/value_bets_log.xlsx
+++ b/data/value_bets_log.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,8 +44,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -87,6 +91,11 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -106,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -133,6 +142,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -500,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1431,6 +1443,2022 @@
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr"/>
     </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>✅ Cameron Norrie</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Jannik Sinner</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="J17" s="10" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>✅ Marko ToPo</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Martin Krumich</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>92.59999999999999</v>
+      </c>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="inlineStr"/>
+      <c r="N18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>✅ Bernard Tomic</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Marat Sharipov</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>TA-hard</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>✅ Hayato Matsuoka</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Keegan Smith</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>45.4</v>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>TA-hard</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="inlineStr"/>
+      <c r="N20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>✅ Pierre-Hugues Herbert</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Pol Martin Tiffon</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>✅ Chun Hsin Tseng</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Lukas Neumayer</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="I22" s="7" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L22" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="inlineStr"/>
+      <c r="N22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>✅ Viktor Durasovic</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Buvaysar Gadamauri</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Shymkent II, Kazakhstan Men Singles</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>✅ Rio Noguchi</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Yu Hsiou Hsu</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="K24" s="7" t="inlineStr">
+        <is>
+          <t>TA-hard</t>
+        </is>
+      </c>
+      <c r="L24" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M24" s="7" t="inlineStr"/>
+      <c r="N24" s="7" t="inlineStr"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>✅ Stefanos Tsitsipas</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Casper Ruud</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>✅ Ioannis Xilas</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Michael Geerts</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="K26" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L26" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M26" s="7" t="inlineStr"/>
+      <c r="N26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>✅ Thomas Faurel</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Inaki Montes-de la Torre</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="I27" s="2" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="J27" s="6" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>✅ Vit Kopriva</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Rafael Jodar</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="I28" s="7" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K28" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L28" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M28" s="7" t="inlineStr"/>
+      <c r="N28" s="7" t="inlineStr"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>✅ Jaime Faria</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Andrea Guerrieri</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="J29" s="6" t="n">
+        <v>25.7</v>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sho Shimabukuro</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Yuta Shimizu</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="I30" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="J30" s="6" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="K30" s="7" t="inlineStr">
+        <is>
+          <t>TA-hard</t>
+        </is>
+      </c>
+      <c r="L30" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M30" s="7" t="inlineStr"/>
+      <c r="N30" s="7" t="inlineStr"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>✅ Frederico Ferreira Silva</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Sanchez Jover</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>70.3</v>
+      </c>
+      <c r="J31" s="6" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>✅ Luka Pavlovic</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Vitaliy Sachko</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I32" s="7" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="J32" s="9" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L32" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M32" s="7" t="inlineStr"/>
+      <c r="N32" s="7" t="inlineStr"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>✅ Dalibor Svrcina</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Felix Gill</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="I33" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="J33" s="9" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>✅ Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Leylah Fernandez</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>WTA - WTA Madrid, Spain Women Singles</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I34" s="7" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="J34" s="9" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L34" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M34" s="7" t="inlineStr"/>
+      <c r="N34" s="7" t="inlineStr"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>✅ Tom Paris</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Sascha Gueymard Wayenburg</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="I35" s="2" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="J35" s="9" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>✅ Matteo Berrettini</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Patrick Kypson</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H36" s="5" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="I36" s="7" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="J36" s="9" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L36" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M36" s="7" t="inlineStr"/>
+      <c r="N36" s="7" t="inlineStr"/>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>✅ Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Jakub Mensik</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="J37" s="9" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr"/>
+      <c r="N37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>✅ Lorenzo Musetti</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Jiri Lehecka</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="I38" s="7" t="n">
+        <v>69.2</v>
+      </c>
+      <c r="J38" s="9" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L38" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M38" s="7" t="inlineStr"/>
+      <c r="N38" s="7" t="inlineStr"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>✅ Zdenek Kolar</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Filip Cristian Jianu</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="H39" s="5" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="J39" s="9" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>✅ Daniil Medvedev</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Flavio Cobolli</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="I40" s="7" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="J40" s="9" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="K40" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L40" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M40" s="7" t="inlineStr"/>
+      <c r="N40" s="7" t="inlineStr"/>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>✅ Nikoloz Basilashvili</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Sandro Kopp</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H41" s="5" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="I41" s="2" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="J41" s="9" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>✅ Stefanos Sakellaridis</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Enrico Dalla Valle</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="H42" s="5" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="I42" s="7" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="J42" s="9" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L42" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M42" s="7" t="inlineStr"/>
+      <c r="N42" s="7" t="inlineStr"/>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>✅ Adam Walton</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Jie Cui</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H43" s="5" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="I43" s="2" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="J43" s="2" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>TA-hard</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr"/>
+      <c r="N43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>✅ Toby Samuel</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Raul Brancaccio</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="I44" s="7" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="J44" s="7" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L44" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M44" s="7" t="inlineStr"/>
+      <c r="N44" s="7" t="inlineStr"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>✅ Mikhail Kukushkin</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Coleman Wong</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="I45" s="2" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="J45" s="2" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>TA-hard</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr"/>
+      <c r="N45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>✅ Kimmer Coppejans</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Matteo Martineau</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="I46" s="7" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="J46" s="7" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="K46" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L46" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M46" s="7" t="inlineStr"/>
+      <c r="N46" s="7" t="inlineStr"/>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>✅ Tomas Martin Etcheverry</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Arthur Fils</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="H47" s="5" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="I47" s="2" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="J47" s="2" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="inlineStr"/>
+      <c r="N47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>✅ Fajing Sun</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>Tristan Schoolkate</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="H48" s="5" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="I48" s="7" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="J48" s="7" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="K48" s="7" t="inlineStr">
+        <is>
+          <t>TA-hard</t>
+        </is>
+      </c>
+      <c r="L48" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M48" s="7" t="inlineStr"/>
+      <c r="N48" s="7" t="inlineStr"/>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>✅ Norbert Gombos</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Thiago Seyboth Wild</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="H49" s="5" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="I49" s="2" t="n">
+        <v>47.9</v>
+      </c>
+      <c r="J49" s="2" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr"/>
+      <c r="N49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>✅ Ioannis Xilas</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Michael Geerts</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="H50" s="5" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="J50" s="6" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr"/>
+      <c r="N50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>✅ Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Jakub Mensik</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G51" s="8" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="H51" s="5" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="I51" s="7" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="J51" s="9" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="K51" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L51" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M51" s="7" t="inlineStr"/>
+      <c r="N51" s="7" t="inlineStr"/>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>16:29</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>✅ Daniil Medvedev</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Flavio Cobolli</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H52" s="5" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="I52" s="2" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="J52" s="2" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr"/>
+      <c r="N52" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix EV con quota mercato reale e quota equa Elo corretta
</commit_message>
<xml_diff>
--- a/data/value_bets_log.xlsx
+++ b/data/value_bets_log.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3459,6 +3459,566 @@
       <c r="M52" s="2" t="inlineStr"/>
       <c r="N52" s="2" t="inlineStr"/>
     </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>✅ Ioannis Xilas</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Michael Geerts</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="H53" s="5" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="I53" s="2" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="J53" s="10" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr"/>
+      <c r="N53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>✅ Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>Jakub Mensik</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G54" s="8" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="H54" s="5" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="I54" s="7" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="J54" s="9" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="K54" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L54" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M54" s="7" t="inlineStr"/>
+      <c r="N54" s="7" t="inlineStr"/>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>✅ Daniil Medvedev</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Flavio Cobolli</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H55" s="5" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="I55" s="2" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="J55" s="9" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr"/>
+      <c r="N55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>✅ Zachary Svajda</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Hubert Hurkacz</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G56" s="8" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="H56" s="5" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="I56" s="7" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="J56" s="7" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="K56" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L56" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M56" s="7" t="inlineStr"/>
+      <c r="N56" s="7" t="inlineStr"/>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>✅ Cristian Garin</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Moez Echargui</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="H57" s="5" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="I57" s="2" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="J57" s="2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>✅ Michael Mmoh</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Andrew Fenty</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G58" s="8" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="H58" s="5" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="I58" s="7" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="J58" s="7" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="K58" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L58" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M58" s="7" t="inlineStr"/>
+      <c r="N58" s="7" t="inlineStr"/>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>✅ Aryna Sabalenka</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Hailey Baptiste</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>WTA - WTA Madrid, Spain Women Singles</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H59" s="5" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="I59" s="2" t="n">
+        <v>93.3</v>
+      </c>
+      <c r="J59" s="2" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>✅ Ioannis Xilas</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Michael Geerts</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="H60" s="5" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="J60" s="6" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr"/>
+      <c r="N60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>✅ Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>Jakub Mensik</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G61" s="8" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="H61" s="5" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="I61" s="7" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="J61" s="9" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="K61" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L61" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M61" s="7" t="inlineStr"/>
+      <c r="N61" s="7" t="inlineStr"/>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>✅ Daniil Medvedev</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Flavio Cobolli</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H62" s="5" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="I62" s="2" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="J62" s="2" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Forma recente 60 giorni da Tennisexplorer, dati 2026 aggiornati
</commit_message>
<xml_diff>
--- a/data/value_bets_log.xlsx
+++ b/data/value_bets_log.xlsx
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N62"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4019,6 +4019,174 @@
       <c r="M62" s="2" t="inlineStr"/>
       <c r="N62" s="2" t="inlineStr"/>
     </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>✅ Ioannis Xilas</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Michael Geerts</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="H63" s="5" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="I63" s="2" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="J63" s="6" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>✅ Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>Jakub Mensik</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G64" s="8" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="H64" s="5" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="I64" s="7" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="J64" s="9" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="K64" s="7" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L64" s="7" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M64" s="7" t="inlineStr"/>
+      <c r="N64" s="7" t="inlineStr"/>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>✅ Daniil Medvedev</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Flavio Cobolli</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H65" s="5" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="J65" s="2" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>TA-clay</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr"/>
+      <c r="N65" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scanner anticipa partite 1-4 giorni, forma+fatica attivi
</commit_message>
<xml_diff>
--- a/data/value_bets_log.xlsx
+++ b/data/value_bets_log.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,8 +30,22 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +72,46 @@
         <fgColor rgb="0070AD47"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -77,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -89,6 +143,36 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -456,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -565,6 +649,921 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>✅ Hamish Stewart</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Blaise Bicknell</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="H2" s="8" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M2" s="7" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="N2" s="10" t="inlineStr"/>
+      <c r="O2" s="11" t="inlineStr"/>
+      <c r="P2" s="5" t="inlineStr"/>
+      <c r="Q2" s="5" t="inlineStr"/>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>✅ Marcelo Tomas Barrios Vera</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Lukas Neumayer</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="I3" s="12" t="n">
+        <v>67.40000000000001</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="K3" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M3" s="13" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="N3" s="10" t="inlineStr"/>
+      <c r="O3" s="11" t="inlineStr"/>
+      <c r="P3" s="12" t="inlineStr"/>
+      <c r="Q3" s="12" t="inlineStr"/>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>✅ David Goffin</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Thomas Faurel</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="N4" s="10" t="inlineStr"/>
+      <c r="O4" s="11" t="inlineStr"/>
+      <c r="P4" s="5" t="inlineStr"/>
+      <c r="Q4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>✅ Adrian Mannarino</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Jesper De Jong</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="I5" s="12" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M5" s="13" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="N5" s="10" t="inlineStr"/>
+      <c r="O5" s="11" t="inlineStr"/>
+      <c r="P5" s="12" t="inlineStr"/>
+      <c r="Q5" s="12" t="inlineStr"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>✅ David Jorda Sanchis</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Sandro Kopp</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(0.0/-0.3)</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="N6" s="10" t="inlineStr"/>
+      <c r="O6" s="11" t="inlineStr"/>
+      <c r="P6" s="5" t="inlineStr"/>
+      <c r="Q6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>✅ Rudolf Molleker</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Henri Squire</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="K7" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="L7" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M7" s="13" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="N7" s="10" t="inlineStr"/>
+      <c r="O7" s="11" t="inlineStr"/>
+      <c r="P7" s="12" t="inlineStr"/>
+      <c r="Q7" s="12" t="inlineStr"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>✅ Jonas Forejtek</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Zdenek Kolar</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="8" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(0.0/-0.3)</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" s="10" t="inlineStr"/>
+      <c r="O8" s="11" t="inlineStr"/>
+      <c r="P8" s="5" t="inlineStr"/>
+      <c r="Q8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>✅ Arthur Fils</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Jiri Lehecka</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="I9" s="12" t="n">
+        <v>73.8</v>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M9" s="13" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="N9" s="10" t="inlineStr"/>
+      <c r="O9" s="11" t="inlineStr"/>
+      <c r="P9" s="12" t="inlineStr"/>
+      <c r="Q9" s="12" t="inlineStr"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>✅ Jaime Faria</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Martin Krumich</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="J10" s="14" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N10" s="10" t="inlineStr"/>
+      <c r="O10" s="11" t="inlineStr"/>
+      <c r="P10" s="5" t="inlineStr"/>
+      <c r="Q10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>✅ Damir Dzumhur</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Emilio Nava</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="I11" s="12" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="J11" s="14" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="K11" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L11" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M11" s="13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N11" s="10" t="inlineStr"/>
+      <c r="O11" s="11" t="inlineStr"/>
+      <c r="P11" s="12" t="inlineStr"/>
+      <c r="Q11" s="12" t="inlineStr"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>✅ Mert Alkaya</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Paul Jubb</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J12" s="14" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="N12" s="10" t="inlineStr"/>
+      <c r="O12" s="11" t="inlineStr"/>
+      <c r="P12" s="5" t="inlineStr"/>
+      <c r="Q12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>✅ Lorenzo Sonego</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Mattia Bellucci</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I13" s="12" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="J13" s="14" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="K13" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L13" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M13" s="13" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="N13" s="10" t="inlineStr"/>
+      <c r="O13" s="11" t="inlineStr"/>
+      <c r="P13" s="12" t="inlineStr"/>
+      <c r="Q13" s="12" t="inlineStr"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>✅ Vitaliy Sachko</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Nikolas Sanchez Izquierdo</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="J14" s="5" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="N14" s="10" t="inlineStr"/>
+      <c r="O14" s="11" t="inlineStr"/>
+      <c r="P14" s="5" t="inlineStr"/>
+      <c r="Q14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>✅ Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Hailey Baptiste</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>WTA - WTA Madrid, Spain Women Singles</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="I15" s="12" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="K15" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="L15" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N15" s="10" t="inlineStr"/>
+      <c r="O15" s="11" t="inlineStr"/>
+      <c r="P15" s="12" t="inlineStr"/>
+      <c r="Q15" s="12" t="inlineStr"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>✅ Adam Walton</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Jie Cui</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="H16" s="8" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="J16" s="5" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>TA-hard+forma</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M16" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="N16" s="10" t="inlineStr"/>
+      <c r="O16" s="11" t="inlineStr"/>
+      <c r="P16" s="5" t="inlineStr"/>
+      <c r="Q16" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Data partita corretta nell'Excel, field data_partita propagato
</commit_message>
<xml_diff>
--- a/data/value_bets_log.xlsx
+++ b/data/value_bets_log.xlsx
@@ -540,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1564,6 +1564,1714 @@
       <c r="P16" s="5" t="inlineStr"/>
       <c r="Q16" s="5" t="inlineStr"/>
     </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>✅ David Goffin</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Thomas Faurel</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="J17" s="9" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="N17" s="10" t="inlineStr"/>
+      <c r="O17" s="11" t="inlineStr"/>
+      <c r="P17" s="5" t="inlineStr"/>
+      <c r="Q17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>✅ Adrian Mannarino</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Jesper De Jong</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="I18" s="12" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="J18" s="9" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="K18" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L18" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M18" s="13" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="N18" s="10" t="inlineStr"/>
+      <c r="O18" s="11" t="inlineStr"/>
+      <c r="P18" s="12" t="inlineStr"/>
+      <c r="Q18" s="12" t="inlineStr"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>✅ David Jorda Sanchis</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Sandro Kopp</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="J19" s="9" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(0.0/-0.3)</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="N19" s="10" t="inlineStr"/>
+      <c r="O19" s="11" t="inlineStr"/>
+      <c r="P19" s="5" t="inlineStr"/>
+      <c r="Q19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>✅ Rudolf Molleker</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Henri Squire</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G20" s="13" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="H20" s="8" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="I20" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="K20" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="L20" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M20" s="13" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="N20" s="10" t="inlineStr"/>
+      <c r="O20" s="11" t="inlineStr"/>
+      <c r="P20" s="12" t="inlineStr"/>
+      <c r="Q20" s="12" t="inlineStr"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>✅ Jonas Forejtek</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Zdenek Kolar</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="J21" s="14" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(0.0/-0.3)</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N21" s="10" t="inlineStr"/>
+      <c r="O21" s="11" t="inlineStr"/>
+      <c r="P21" s="5" t="inlineStr"/>
+      <c r="Q21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>✅ Arthur Fils</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Jiri Lehecka</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="H22" s="8" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="I22" s="12" t="n">
+        <v>73.8</v>
+      </c>
+      <c r="J22" s="14" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="K22" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L22" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M22" s="13" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="N22" s="10" t="inlineStr"/>
+      <c r="O22" s="11" t="inlineStr"/>
+      <c r="P22" s="12" t="inlineStr"/>
+      <c r="Q22" s="12" t="inlineStr"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>✅ Jaime Faria</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Martin Krumich</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="J23" s="14" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N23" s="10" t="inlineStr"/>
+      <c r="O23" s="11" t="inlineStr"/>
+      <c r="P23" s="5" t="inlineStr"/>
+      <c r="Q23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>✅ Damir Dzumhur</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Emilio Nava</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H24" s="8" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="I24" s="12" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="J24" s="14" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="K24" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L24" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M24" s="13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N24" s="10" t="inlineStr"/>
+      <c r="O24" s="11" t="inlineStr"/>
+      <c r="P24" s="12" t="inlineStr"/>
+      <c r="Q24" s="12" t="inlineStr"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>✅ Mert Alkaya</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Paul Jubb</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J25" s="14" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="N25" s="10" t="inlineStr"/>
+      <c r="O25" s="11" t="inlineStr"/>
+      <c r="P25" s="5" t="inlineStr"/>
+      <c r="Q25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>✅ Lorenzo Sonego</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Mattia Bellucci</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G26" s="13" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="H26" s="8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I26" s="12" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="J26" s="14" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="K26" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L26" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M26" s="13" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="N26" s="10" t="inlineStr"/>
+      <c r="O26" s="11" t="inlineStr"/>
+      <c r="P26" s="12" t="inlineStr"/>
+      <c r="Q26" s="12" t="inlineStr"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>✅ Vitaliy Sachko</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Nikolas Sanchez Izquierdo</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="J27" s="5" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="N27" s="10" t="inlineStr"/>
+      <c r="O27" s="11" t="inlineStr"/>
+      <c r="P27" s="5" t="inlineStr"/>
+      <c r="Q27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>✅ Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>Hailey Baptiste</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>WTA - WTA Madrid, Spain Women Singles</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G28" s="13" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H28" s="8" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="J28" s="12" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="K28" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="L28" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M28" s="13" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N28" s="10" t="inlineStr"/>
+      <c r="O28" s="11" t="inlineStr"/>
+      <c r="P28" s="12" t="inlineStr"/>
+      <c r="Q28" s="12" t="inlineStr"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>✅ Adam Walton</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Jie Cui</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="H29" s="8" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="J29" s="5" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>TA-hard+forma</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="N29" s="10" t="inlineStr"/>
+      <c r="O29" s="11" t="inlineStr"/>
+      <c r="P29" s="5" t="inlineStr"/>
+      <c r="Q29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>✅ Hamish Stewart</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Blaise Bicknell</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="H30" s="8" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="I30" s="12" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="J30" s="12" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="K30" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L30" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M30" s="13" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="N30" s="10" t="inlineStr"/>
+      <c r="O30" s="11" t="inlineStr"/>
+      <c r="P30" s="12" t="inlineStr"/>
+      <c r="Q30" s="12" t="inlineStr"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>✅ David Goffin</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Thomas Faurel</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="H31" s="8" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="J31" s="9" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="N31" s="10" t="inlineStr"/>
+      <c r="O31" s="11" t="inlineStr"/>
+      <c r="P31" s="5" t="inlineStr"/>
+      <c r="Q31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>✅ Adrian Mannarino</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>Jesper De Jong</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G32" s="13" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="H32" s="8" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="I32" s="12" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="J32" s="9" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="K32" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L32" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M32" s="13" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="N32" s="10" t="inlineStr"/>
+      <c r="O32" s="11" t="inlineStr"/>
+      <c r="P32" s="12" t="inlineStr"/>
+      <c r="Q32" s="12" t="inlineStr"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>✅ David Jorda Sanchis</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Sandro Kopp</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="H33" s="8" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="J33" s="9" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(0.0/-0.3)</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M33" s="7" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="N33" s="10" t="inlineStr"/>
+      <c r="O33" s="11" t="inlineStr"/>
+      <c r="P33" s="5" t="inlineStr"/>
+      <c r="Q33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>✅ Rudolf Molleker</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>Henri Squire</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="H34" s="8" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="I34" s="12" t="n">
+        <v>48</v>
+      </c>
+      <c r="J34" s="9" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="K34" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="L34" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M34" s="13" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="N34" s="10" t="inlineStr"/>
+      <c r="O34" s="11" t="inlineStr"/>
+      <c r="P34" s="12" t="inlineStr"/>
+      <c r="Q34" s="12" t="inlineStr"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>✅ Jonas Forejtek</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Zdenek Kolar</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" s="8" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="J35" s="14" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(0.0/-0.3)</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M35" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N35" s="10" t="inlineStr"/>
+      <c r="O35" s="11" t="inlineStr"/>
+      <c r="P35" s="5" t="inlineStr"/>
+      <c r="Q35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>✅ Arthur Fils</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>Jiri Lehecka</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G36" s="13" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="H36" s="8" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="I36" s="12" t="n">
+        <v>73.8</v>
+      </c>
+      <c r="J36" s="14" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="K36" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L36" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M36" s="13" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="N36" s="10" t="inlineStr"/>
+      <c r="O36" s="11" t="inlineStr"/>
+      <c r="P36" s="12" t="inlineStr"/>
+      <c r="Q36" s="12" t="inlineStr"/>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>✅ Jaime Faria</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Martin Krumich</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H37" s="8" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="I37" s="5" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="J37" s="14" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M37" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N37" s="10" t="inlineStr"/>
+      <c r="O37" s="11" t="inlineStr"/>
+      <c r="P37" s="5" t="inlineStr"/>
+      <c r="Q37" s="5" t="inlineStr"/>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>✅ Damir Dzumhur</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>Emilio Nava</t>
+        </is>
+      </c>
+      <c r="E38" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G38" s="13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H38" s="8" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="I38" s="12" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="J38" s="14" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="K38" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L38" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M38" s="13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N38" s="10" t="inlineStr"/>
+      <c r="O38" s="11" t="inlineStr"/>
+      <c r="P38" s="12" t="inlineStr"/>
+      <c r="Q38" s="12" t="inlineStr"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>✅ Mert Alkaya</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Paul Jubb</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H39" s="8" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="J39" s="14" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="N39" s="10" t="inlineStr"/>
+      <c r="O39" s="11" t="inlineStr"/>
+      <c r="P39" s="5" t="inlineStr"/>
+      <c r="Q39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>✅ Lorenzo Sonego</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
+        <is>
+          <t>Mattia Bellucci</t>
+        </is>
+      </c>
+      <c r="E40" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G40" s="13" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="H40" s="8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I40" s="12" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="J40" s="14" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="K40" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L40" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M40" s="13" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="N40" s="10" t="inlineStr"/>
+      <c r="O40" s="11" t="inlineStr"/>
+      <c r="P40" s="12" t="inlineStr"/>
+      <c r="Q40" s="12" t="inlineStr"/>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>✅ Vitaliy Sachko</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Nikolas Sanchez Izquierdo</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="H41" s="8" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="I41" s="5" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="J41" s="5" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M41" s="7" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="N41" s="10" t="inlineStr"/>
+      <c r="O41" s="11" t="inlineStr"/>
+      <c r="P41" s="5" t="inlineStr"/>
+      <c r="Q41" s="5" t="inlineStr"/>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>✅ Mirra Andreeva</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>Hailey Baptiste</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="inlineStr">
+        <is>
+          <t>WTA - WTA Madrid, Spain Women Singles</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G42" s="13" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H42" s="8" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="I42" s="12" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="J42" s="12" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="K42" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="L42" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M42" s="13" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N42" s="10" t="inlineStr"/>
+      <c r="O42" s="11" t="inlineStr"/>
+      <c r="P42" s="12" t="inlineStr"/>
+      <c r="Q42" s="12" t="inlineStr"/>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>✅ Adam Walton</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Jie Cui</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="H43" s="8" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="I43" s="5" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="J43" s="5" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>TA-hard+forma</t>
+        </is>
+      </c>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M43" s="7" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="N43" s="10" t="inlineStr"/>
+      <c r="O43" s="11" t="inlineStr"/>
+      <c r="P43" s="5" t="inlineStr"/>
+      <c r="Q43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>✅ Hamish Stewart</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>Blaise Bicknell</t>
+        </is>
+      </c>
+      <c r="E44" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G44" s="13" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="H44" s="8" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="I44" s="12" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="J44" s="12" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="K44" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L44" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M44" s="13" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="N44" s="10" t="inlineStr"/>
+      <c r="O44" s="11" t="inlineStr"/>
+      <c r="P44" s="12" t="inlineStr"/>
+      <c r="Q44" s="12" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix get_quote_handicap_evento - chiave hdp e Spread Games, Scanner B operativo
</commit_message>
<xml_diff>
--- a/data/value_bets_log.xlsx
+++ b/data/value_bets_log.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Value Bets Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Handicap Bets" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -45,7 +46,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -112,6 +113,11 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E4E79"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -131,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -173,6 +179,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3275,4 +3284,106 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>Ora</t>
+        </is>
+      </c>
+      <c r="C1" s="15" t="inlineStr">
+        <is>
+          <t>Punta su (handicap)</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>Avversario</t>
+        </is>
+      </c>
+      <c r="E1" s="15" t="inlineStr">
+        <is>
+          <t>Handicap</t>
+        </is>
+      </c>
+      <c r="F1" s="15" t="inlineStr">
+        <is>
+          <t>Quota</t>
+        </is>
+      </c>
+      <c r="G1" s="15" t="inlineStr">
+        <is>
+          <t>Prob %</t>
+        </is>
+      </c>
+      <c r="H1" s="15" t="inlineStr">
+        <is>
+          <t>EV %</t>
+        </is>
+      </c>
+      <c r="I1" s="15" t="inlineStr">
+        <is>
+          <t>Torneo</t>
+        </is>
+      </c>
+      <c r="J1" s="15" t="inlineStr">
+        <is>
+          <t>Superficie</t>
+        </is>
+      </c>
+      <c r="K1" s="15" t="inlineStr">
+        <is>
+          <t>Elo Diff</t>
+        </is>
+      </c>
+      <c r="L1" s="15" t="inlineStr">
+        <is>
+          <t>Margine Atteso</t>
+        </is>
+      </c>
+      <c r="M1" s="15" t="inlineStr">
+        <is>
+          <t>Elo Usato</t>
+        </is>
+      </c>
+      <c r="N1" s="15" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
main.py unifica Scanner A ML e Scanner B Handicap in un unico comando
</commit_message>
<xml_diff>
--- a/data/value_bets_log.xlsx
+++ b/data/value_bets_log.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,8 +45,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -118,6 +122,16 @@
         <fgColor rgb="001E4E79"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEEFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -137,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -182,6 +196,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -549,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q44"/>
+  <dimension ref="A1:Q63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -838,8 +861,14 @@
       </c>
       <c r="N4" s="10" t="inlineStr"/>
       <c r="O4" s="11" t="inlineStr"/>
-      <c r="P4" s="5" t="inlineStr"/>
-      <c r="Q4" s="5" t="inlineStr"/>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
@@ -1021,8 +1050,14 @@
       </c>
       <c r="N7" s="10" t="inlineStr"/>
       <c r="O7" s="11" t="inlineStr"/>
-      <c r="P7" s="12" t="inlineStr"/>
-      <c r="Q7" s="12" t="inlineStr"/>
+      <c r="P7" s="12" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="Q7" s="12" t="n">
+        <v>1.52</v>
+      </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -1143,8 +1178,14 @@
       </c>
       <c r="N9" s="10" t="inlineStr"/>
       <c r="O9" s="11" t="inlineStr"/>
-      <c r="P9" s="12" t="inlineStr"/>
-      <c r="Q9" s="12" t="inlineStr"/>
+      <c r="P9" s="12" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="Q9" s="12" t="n">
+        <v>0.57</v>
+      </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -1265,8 +1306,14 @@
       </c>
       <c r="N11" s="10" t="inlineStr"/>
       <c r="O11" s="11" t="inlineStr"/>
-      <c r="P11" s="12" t="inlineStr"/>
-      <c r="Q11" s="12" t="inlineStr"/>
+      <c r="P11" s="12" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="Q11" s="12" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -1326,8 +1373,14 @@
       </c>
       <c r="N12" s="10" t="inlineStr"/>
       <c r="O12" s="11" t="inlineStr"/>
-      <c r="P12" s="5" t="inlineStr"/>
-      <c r="Q12" s="5" t="inlineStr"/>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="n">
+        <v>1.1</v>
+      </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
@@ -1387,8 +1440,14 @@
       </c>
       <c r="N13" s="10" t="inlineStr"/>
       <c r="O13" s="11" t="inlineStr"/>
-      <c r="P13" s="12" t="inlineStr"/>
-      <c r="Q13" s="12" t="inlineStr"/>
+      <c r="P13" s="12" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="Q13" s="12" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -1570,8 +1629,14 @@
       </c>
       <c r="N16" s="10" t="inlineStr"/>
       <c r="O16" s="11" t="inlineStr"/>
-      <c r="P16" s="5" t="inlineStr"/>
-      <c r="Q16" s="5" t="inlineStr"/>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="n">
+        <v>0.27</v>
+      </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -3280,6 +3345,1165 @@
       <c r="O44" s="11" t="inlineStr"/>
       <c r="P44" s="12" t="inlineStr"/>
       <c r="Q44" s="12" t="inlineStr"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>✅ Alexander Binda</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Manas Dhamne</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Shymkent II, Kazakhstan Men Singles</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H45" s="8" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="I45" s="5" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="J45" s="18" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M45" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="N45" s="10" t="inlineStr"/>
+      <c r="O45" s="11" t="inlineStr"/>
+      <c r="P45" s="5" t="inlineStr"/>
+      <c r="Q45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>✅ Kimmer Coppejans</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="inlineStr">
+        <is>
+          <t>Pol Martin Tiffon</t>
+        </is>
+      </c>
+      <c r="E46" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="F46" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G46" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H46" s="8" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="I46" s="12" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="J46" s="9" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="K46" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="L46" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M46" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="N46" s="10" t="inlineStr"/>
+      <c r="O46" s="11" t="inlineStr"/>
+      <c r="P46" s="12" t="inlineStr"/>
+      <c r="Q46" s="12" t="inlineStr"/>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>✅ Rinky Hijikata</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Zizou Bergs</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="H47" s="8" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="I47" s="5" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="J47" s="9" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(0.0/-0.3)</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M47" s="7" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="N47" s="10" t="inlineStr"/>
+      <c r="O47" s="11" t="inlineStr"/>
+      <c r="P47" s="5" t="inlineStr"/>
+      <c r="Q47" s="5" t="inlineStr"/>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>✅ Laslo Djere</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>Lukas Neumayer</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G48" s="13" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H48" s="8" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="I48" s="12" t="n">
+        <v>74.3</v>
+      </c>
+      <c r="J48" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="K48" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="L48" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M48" s="13" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="N48" s="10" t="inlineStr"/>
+      <c r="O48" s="11" t="inlineStr"/>
+      <c r="P48" s="12" t="inlineStr"/>
+      <c r="Q48" s="12" t="inlineStr"/>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>✅ Alex Bolt</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Keegan Smith</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="H49" s="8" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="I49" s="5" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="J49" s="9" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>TA-hard+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M49" s="7" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="N49" s="10" t="inlineStr"/>
+      <c r="O49" s="11" t="inlineStr"/>
+      <c r="P49" s="5" t="inlineStr"/>
+      <c r="Q49" s="5" t="inlineStr"/>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>✅ Marcos Giron</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>Roman Andres Burruchaga</t>
+        </is>
+      </c>
+      <c r="E50" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G50" s="13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H50" s="8" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="I50" s="12" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="J50" s="9" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="K50" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L50" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M50" s="13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N50" s="10" t="inlineStr"/>
+      <c r="O50" s="11" t="inlineStr"/>
+      <c r="P50" s="12" t="inlineStr"/>
+      <c r="Q50" s="12" t="inlineStr"/>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>✅ Matteo Arnaldi</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Nuno Borges</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H51" s="8" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="I51" s="5" t="n">
+        <v>57.7</v>
+      </c>
+      <c r="J51" s="9" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="K51" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M51" s="7" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="N51" s="10" t="inlineStr"/>
+      <c r="O51" s="11" t="inlineStr"/>
+      <c r="P51" s="5" t="inlineStr"/>
+      <c r="Q51" s="5" t="inlineStr"/>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>✅ Mert Alkaya</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>Gauthier Onclin</t>
+        </is>
+      </c>
+      <c r="E52" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F52" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G52" s="13" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="H52" s="8" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="I52" s="12" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="J52" s="14" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="K52" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="L52" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M52" s="13" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="N52" s="10" t="inlineStr"/>
+      <c r="O52" s="11" t="inlineStr"/>
+      <c r="P52" s="12" t="inlineStr"/>
+      <c r="Q52" s="12" t="inlineStr"/>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>✅ Hamish Stewart</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Eliakim Coulibaly</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="H53" s="8" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="I53" s="5" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="J53" s="14" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="K53" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M53" s="7" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="N53" s="10" t="inlineStr"/>
+      <c r="O53" s="11" t="inlineStr"/>
+      <c r="P53" s="5" t="inlineStr"/>
+      <c r="Q53" s="5" t="inlineStr"/>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>✅ Mili Poljicak</t>
+        </is>
+      </c>
+      <c r="D54" s="12" t="inlineStr">
+        <is>
+          <t>Buvaysar Gadamauri</t>
+        </is>
+      </c>
+      <c r="E54" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Shymkent II, Kazakhstan Men Singles</t>
+        </is>
+      </c>
+      <c r="F54" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G54" s="13" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="H54" s="8" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="I54" s="12" t="n">
+        <v>75.7</v>
+      </c>
+      <c r="J54" s="14" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="K54" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L54" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M54" s="13" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="N54" s="10" t="inlineStr"/>
+      <c r="O54" s="11" t="inlineStr"/>
+      <c r="P54" s="12" t="inlineStr"/>
+      <c r="Q54" s="12" t="inlineStr"/>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>✅ Antoine Ghibaudo</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Andrej Nedic</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Shymkent II, Kazakhstan Men Singles</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="H55" s="8" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="I55" s="5" t="n">
+        <v>41.8</v>
+      </c>
+      <c r="J55" s="14" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="K55" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="L55" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M55" s="7" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="N55" s="10" t="inlineStr"/>
+      <c r="O55" s="11" t="inlineStr"/>
+      <c r="P55" s="5" t="inlineStr"/>
+      <c r="Q55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>✅ Arthur Fils</t>
+        </is>
+      </c>
+      <c r="D56" s="12" t="inlineStr">
+        <is>
+          <t>Jannik Sinner</t>
+        </is>
+      </c>
+      <c r="E56" s="12" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F56" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G56" s="13" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="H56" s="8" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="I56" s="12" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="J56" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="K56" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="L56" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M56" s="13" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="N56" s="10" t="inlineStr"/>
+      <c r="O56" s="11" t="inlineStr"/>
+      <c r="P56" s="12" t="inlineStr"/>
+      <c r="Q56" s="12" t="inlineStr"/>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>✅ Yibing Wu</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Ethan Quinn</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H57" s="8" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="I57" s="5" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="J57" s="14" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="K57" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M57" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="N57" s="10" t="inlineStr"/>
+      <c r="O57" s="11" t="inlineStr"/>
+      <c r="P57" s="5" t="inlineStr"/>
+      <c r="Q57" s="5" t="inlineStr"/>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>✅ Fajing Sun</t>
+        </is>
+      </c>
+      <c r="D58" s="12" t="inlineStr">
+        <is>
+          <t>Mark Lajal</t>
+        </is>
+      </c>
+      <c r="E58" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="F58" s="12" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="G58" s="13" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="H58" s="8" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="I58" s="12" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="J58" s="14" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="K58" s="12" t="inlineStr">
+        <is>
+          <t>TA-hard+forma+fat(0.0/-0.3)</t>
+        </is>
+      </c>
+      <c r="L58" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M58" s="13" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="N58" s="10" t="inlineStr"/>
+      <c r="O58" s="11" t="inlineStr"/>
+      <c r="P58" s="12" t="inlineStr"/>
+      <c r="Q58" s="12" t="inlineStr"/>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>✅ Jesper De Jong</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Gianluca Cadenasso</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="H59" s="8" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="I59" s="5" t="n">
+        <v>69.8</v>
+      </c>
+      <c r="J59" s="5" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="K59" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="L59" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M59" s="7" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="N59" s="10" t="inlineStr"/>
+      <c r="O59" s="11" t="inlineStr"/>
+      <c r="P59" s="5" t="inlineStr"/>
+      <c r="Q59" s="5" t="inlineStr"/>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>✅ Jaime Faria</t>
+        </is>
+      </c>
+      <c r="D60" s="12" t="inlineStr">
+        <is>
+          <t>Miguel Damas</t>
+        </is>
+      </c>
+      <c r="E60" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F60" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G60" s="13" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="H60" s="8" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="I60" s="12" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="J60" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="K60" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L60" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M60" s="13" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="N60" s="10" t="inlineStr"/>
+      <c r="O60" s="11" t="inlineStr"/>
+      <c r="P60" s="12" t="inlineStr"/>
+      <c r="Q60" s="12" t="inlineStr"/>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>✅ Roman Safiullin</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>David Jorda Sanchis</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H61" s="8" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="I61" s="5" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="J61" s="5" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="K61" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L61" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M61" s="7" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="N61" s="10" t="inlineStr"/>
+      <c r="O61" s="11" t="inlineStr"/>
+      <c r="P61" s="5" t="inlineStr"/>
+      <c r="Q61" s="5" t="inlineStr"/>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>✅ Alexander Zverev</t>
+        </is>
+      </c>
+      <c r="D62" s="12" t="inlineStr">
+        <is>
+          <t>Alexander Blockx</t>
+        </is>
+      </c>
+      <c r="E62" s="12" t="inlineStr">
+        <is>
+          <t>ATP - ATP Madrid, Spain Men Singles</t>
+        </is>
+      </c>
+      <c r="F62" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G62" s="13" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="H62" s="8" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I62" s="12" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="J62" s="12" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="K62" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="L62" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M62" s="13" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="N62" s="10" t="inlineStr"/>
+      <c r="O62" s="11" t="inlineStr"/>
+      <c r="P62" s="12" t="inlineStr"/>
+      <c r="Q62" s="12" t="inlineStr"/>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>02:36</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>✅ Ignacio Buse</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Alejandro Tabilo</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="H63" s="8" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="I63" s="5" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="J63" s="5" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="K63" s="5" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="L63" s="5" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+      <c r="M63" s="7" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="N63" s="10" t="inlineStr"/>
+      <c r="O63" s="11" t="inlineStr"/>
+      <c r="P63" s="5" t="inlineStr"/>
+      <c r="Q63" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3292,7 +4516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3383,6 +4607,1566 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>✅ Kimmer Coppejans  +1.5</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>Pol Martin Tiffon</t>
+        </is>
+      </c>
+      <c r="E2" s="16" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F2" s="17" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G2" s="16" t="n">
+        <v>77.90000000000001</v>
+      </c>
+      <c r="H2" s="18" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="I2" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="J2" s="16" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K2" s="16" t="n">
+        <v>134</v>
+      </c>
+      <c r="L2" s="16" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="M2" s="16" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="N2" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>✅ Kimmer Coppejans  +0.5</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Pol Martin Tiffon</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="G3" s="12" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="H3" s="18" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="J3" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K3" s="12" t="n">
+        <v>134</v>
+      </c>
+      <c r="L3" s="12" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="M3" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="N3" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>✅ Fajing Sun  +2.5</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>Mark Lajal</t>
+        </is>
+      </c>
+      <c r="E4" s="16" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F4" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="16" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="J4" s="16" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="K4" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="L4" s="16" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M4" s="16" t="inlineStr">
+        <is>
+          <t>TA-hard+forma+fat(0.0/-0.3)</t>
+        </is>
+      </c>
+      <c r="N4" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>✅ Mert Alkaya  +3.5</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Gauthier Onclin</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>95</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="M5" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="N5" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>✅ Matteo Arnaldi  +1.5</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>Nuno Borges</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G6" s="16" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="J6" s="16" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K6" s="16" t="n">
+        <v>54</v>
+      </c>
+      <c r="L6" s="16" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="M6" s="16" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="N6" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>✅ Rinky Hijikata  +3.5</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Zizou Bergs</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="L7" s="12" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="M7" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(0.0/-0.3)</t>
+        </is>
+      </c>
+      <c r="N7" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>✅ Alex Bolt  -2.5</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Keegan Smith</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="K8" s="16" t="n">
+        <v>290</v>
+      </c>
+      <c r="L8" s="16" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M8" s="16" t="inlineStr">
+        <is>
+          <t>TA-hard+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="N8" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>✅ Laslo Djere  -1.5</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Lukas Neumayer</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G9" s="12" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>184</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="M9" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="N9" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>✅ Alexis Galarneau  +2.5</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>Adam Walton</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="H10" s="14" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="J10" s="16" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="K10" s="16" t="n">
+        <v>64</v>
+      </c>
+      <c r="L10" s="16" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="M10" s="16" t="inlineStr">
+        <is>
+          <t>TA-hard+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="N10" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>✅ Raul Brancaccio  +2.5</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Marco Cecchinato</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="G11" s="12" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="H11" s="14" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>76</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="M11" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="N11" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>✅ Nerman Fatic  -0.5</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Zdenek Kolar</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K12" s="16" t="n">
+        <v>104</v>
+      </c>
+      <c r="L12" s="16" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="M12" s="16" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="N12" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>✅ Matteo Arnaldi  +0.5</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Nuno Borges</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="G13" s="12" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="H13" s="14" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K13" s="12" t="n">
+        <v>54</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="M13" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="N13" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>✅ Matteo Berrettini  +0.5</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Hubert Hurkacz</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="G14" s="16" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H14" s="14" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K14" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="L14" s="16" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="M14" s="16" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="N14" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>02:37</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>✅ Kimmer Coppejans  +1.5</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Pol Martin Tiffon</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="G15" s="16" t="n">
+        <v>77.90000000000001</v>
+      </c>
+      <c r="H15" s="18" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="n">
+        <v>134</v>
+      </c>
+      <c r="L15" s="16" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="M15" s="16" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="N15" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>02:37</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>✅ Kimmer Coppejans  +0.5</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Pol Martin Tiffon</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="G16" s="12" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="H16" s="18" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>134</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="M16" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>02:37</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>✅ Fajing Sun  +2.5</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Mark Lajal</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="16" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="H17" s="9" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="L17" s="16" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M17" s="16" t="inlineStr">
+        <is>
+          <t>TA-hard+forma+fat(0.0/-0.3)</t>
+        </is>
+      </c>
+      <c r="N17" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>02:37</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>✅ Mert Alkaya  +3.5</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Gauthier Onclin</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G18" s="12" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="H18" s="9" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Abidjan 2, Cote d Ivoire, Men Singles</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>95</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="M18" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>02:37</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>✅ Matteo Arnaldi  +1.5</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Nuno Borges</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F19" s="17" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G19" s="16" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="H19" s="9" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="n">
+        <v>54</v>
+      </c>
+      <c r="L19" s="16" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="M19" s="16" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="N19" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>02:37</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>✅ Rinky Hijikata  +3.5</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Zizou Bergs</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G20" s="12" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Aix en Provence, France Men Singles</t>
+        </is>
+      </c>
+      <c r="J20" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K20" s="12" t="n">
+        <v>81</v>
+      </c>
+      <c r="L20" s="12" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="M20" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(0.0/-0.3)</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>02:37</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>✅ Alex Bolt  -2.5</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Keegan Smith</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="F21" s="17" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G21" s="16" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="n">
+        <v>290</v>
+      </c>
+      <c r="L21" s="16" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M21" s="16" t="inlineStr">
+        <is>
+          <t>TA-hard+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="N21" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>02:37</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>✅ Laslo Djere  -1.5</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Lukas Neumayer</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G22" s="12" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="H22" s="9" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Mauthausen, Austria Men Singles</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K22" s="12" t="n">
+        <v>184</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="M22" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>02:37</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>✅ Alexis Galarneau  +2.5</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Adam Walton</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F23" s="17" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G23" s="16" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="H23" s="14" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Jiujiang, China Men Singles</t>
+        </is>
+      </c>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>HARD</t>
+        </is>
+      </c>
+      <c r="K23" s="16" t="n">
+        <v>64</v>
+      </c>
+      <c r="L23" s="16" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="M23" s="16" t="inlineStr">
+        <is>
+          <t>TA-hard+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="N23" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>02:37</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>✅ Raul Brancaccio  +2.5</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Marco Cecchinato</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="G24" s="12" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K24" s="12" t="n">
+        <v>76</v>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="M24" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/-0.3)</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>02:37</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>✅ Nerman Fatic  -0.5</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Zdenek Kolar</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="F25" s="17" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="G25" s="16" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="H25" s="14" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Ostrava, Czech Republic Men Singles</t>
+        </is>
+      </c>
+      <c r="J25" s="16" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K25" s="16" t="n">
+        <v>104</v>
+      </c>
+      <c r="L25" s="16" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="M25" s="16" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="N25" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>02:37</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>✅ Matteo Arnaldi  +0.5</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Nuno Borges</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="G26" s="12" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="H26" s="14" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="I26" s="12" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="J26" s="12" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K26" s="12" t="n">
+        <v>54</v>
+      </c>
+      <c r="L26" s="12" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="M26" s="12" t="inlineStr">
+        <is>
+          <t>TA-clay+forma+fat(-0.3/0.0)</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>02:37</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>✅ Matteo Berrettini  +0.5</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Hubert Hurkacz</t>
+        </is>
+      </c>
+      <c r="E27" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F27" s="17" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="G27" s="16" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="H27" s="14" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <t>Challenger - ATP Challenger Cagliari, Italy Men Singles</t>
+        </is>
+      </c>
+      <c r="J27" s="16" t="inlineStr">
+        <is>
+          <t>CLAY</t>
+        </is>
+      </c>
+      <c r="K27" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="L27" s="16" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="M27" s="16" t="inlineStr">
+        <is>
+          <t>TA-clay+forma</t>
+        </is>
+      </c>
+      <c r="N27" s="16" t="inlineStr">
+        <is>
+          <t>odds-api.io</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>